<commit_message>
remove deprecated #STATA command
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/test_save.xlsx
+++ b/tests/testthat/excel/test_save.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="36">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -134,9 +134,6 @@
   </si>
   <si>
     <t xml:space="preserve">no</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#STATA</t>
   </si>
 </sst>
 </file>
@@ -239,7 +236,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -339,7 +336,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I28"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -684,7 +681,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -701,16 +698,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A3:C3"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A3"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>5</v>
-      </c>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
remove erroneous named region R_id_var that caused an error with the new version of openxlsx2 (the error was: Error (test-save_mapping.R:2:1): (code run outside of `test_that()`) <dplyr:::mutate_error/rlang_error/error/condition> Error in `mutate(filter(named_regions, grepl("^R_*", .data$name)), data = map_if(map(.x = .data$name,     ~wb_read(mapping$wb, named_region = .x, col_names = FALSE)),     negate(is.null), pull))`: ℹ In argument: `data = map_if(...)`. Caused by error in `map()`: ℹ In index: 1. Caused by error in `wb_to_df()`: ! sheet not found. available sheets are: Variables, Label, Verbatims, Free1 )
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/test_save.xlsx
+++ b/tests/testthat/excel/test_save.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datadaptor\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0934F79-5487-4B47-A5F2-A5C6321F3E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AAB612C-34F9-4FDF-AAC0-4302452A8015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,6 @@
     <sheet name="Verbatims" sheetId="3" r:id="rId3"/>
     <sheet name="Free1" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="R_id_var">Label!#REF!</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">

</xml_diff>